<commit_message>
Completed a full functional verification of the assert feature.
</commit_message>
<xml_diff>
--- a/src/MxDBUnit/resources/mxdbunit/sample/sample1.xlsx
+++ b/src/MxDBUnit/resources/mxdbunit/sample/sample1.xlsx
@@ -8,14 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\MxDBUnit\src\MxDBUnit\resources\mxdbunit\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9839A66A-D615-49B1-8001-FFE7F5CE34E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1C96D9-8470-48B3-89C5-D9F9B73F8BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="48180" yWindow="-636" windowWidth="16908" windowHeight="13416" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37044" yWindow="-12336" windowWidth="22452" windowHeight="12192" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Item" sheetId="1" r:id="rId1"/>
-    <sheet name="Order" sheetId="2" r:id="rId2"/>
-    <sheet name="OrderItem" sheetId="3" r:id="rId3"/>
+    <sheet name="Customer" sheetId="4" r:id="rId2"/>
+    <sheet name="Order" sheetId="2" r:id="rId3"/>
+    <sheet name="OrderItem" sheetId="3" r:id="rId4"/>
+    <sheet name="Expected_Customer" sheetId="5" r:id="rId5"/>
+    <sheet name="Expected_Order" sheetId="6" r:id="rId6"/>
+    <sheet name="Expected_OrderItem" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,8 +30,95 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>suzuki yuta</author>
+  </authors>
+  <commentList>
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{A5BDBE1C-9C28-4574-A5F6-EDE5007078EE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>Please specify it in ISO 8601 format.
+If the time zone is omitted, the setting from SetContextTimeZoneId or SetDefaultTimeZoneId is used.
+Example1: 2025-12-23T04:56:12+01:00</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">Example2: 2025-12-23T04:56:12
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>suzuki yuta</author>
+  </authors>
+  <commentList>
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{512F867A-07E4-4412-A291-905DA2552C7E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>Please specify it in ISO 8601 format with a time zone.
+Example: 2025-12-23T04:56:12+01:00</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="41">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1"/>
@@ -41,10 +132,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>CustomerName</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>Name</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -117,22 +204,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>2026-10-13T00:00:00+01:00</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Customer of Order_001</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Customer of Order_002</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Customer of Order_003</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>OrderItem_001</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -162,6 +233,54 @@
   </si>
   <si>
     <t>OrderItem_Item</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Customer_001</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Customer_002</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Name of Customer_001</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Name of Customer_002</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Address</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Address of Customer_001</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Address of Customer_002</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Order_Customer</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2025-12-23T04:56:12+09:00</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CumulativeSales</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>TotalAtamount</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Amount</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -169,7 +288,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,6 +302,21 @@
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="MS P ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="MS P ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -488,63 +622,63 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="2" max="2" width="13.3984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D2">
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3">
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <v>300</v>
@@ -557,70 +691,56 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A53E7E-2292-455C-86A3-346B7EDF246B}">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AEE99C2-9E27-465E-B6CB-6A2D58F84035}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.8984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5" customWidth="1"/>
+    <col min="4" max="4" width="15.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2">
-        <v>1001</v>
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+        <v>34</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3">
-        <v>1002</v>
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4">
-        <v>1003</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" t="s">
-        <v>25</v>
+        <v>35</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -630,112 +750,504 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A53E7E-2292-455C-86A3-346B7EDF246B}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="15.59765625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2">
+        <v>1001</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3">
+        <v>1002</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4">
+        <v>1003</v>
+      </c>
+      <c r="C4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EC0B6D4-E629-427B-86DA-8D931806A50F}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="14.3984375" customWidth="1"/>
     <col min="2" max="2" width="12.8984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.8984375" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="14.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B2">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
-        <v>17</v>
+      <c r="C2">
+        <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
-        <v>17</v>
+      <c r="C3">
+        <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B4">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
+      <c r="C4">
+        <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
-        <v>18</v>
+      <c r="C5">
+        <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B6">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
-        <v>18</v>
+      <c r="C6">
+        <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B7">
         <v>16</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05855E9E-4A78-4337-A1E6-41A1A78B0F61}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5" customWidth="1"/>
+    <col min="4" max="4" width="15.69921875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2">
+        <v>7400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3">
+        <v>9200</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A7D26DE-4B43-4B1A-96E5-470F26423CE2}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="15.59765625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2">
+        <v>1001</v>
+      </c>
+      <c r="C2" t="s">
         <v>19</v>
       </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2">
+        <v>7400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3">
+        <v>1002</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3">
+        <v>4400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4">
+        <v>1003</v>
+      </c>
+      <c r="C4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4">
+        <v>4800</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA993482-7DB0-4E07-A12A-DB0076CC842D}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="14.3984375" customWidth="1"/>
+    <col min="2" max="2" width="12.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.8984375" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="14.796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>1100</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3">
+        <v>12</v>
+      </c>
+      <c r="C3">
+        <v>2400</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4">
+        <v>13</v>
+      </c>
+      <c r="C4">
+        <v>3900</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5">
+        <v>14</v>
+      </c>
+      <c r="C5">
+        <v>1400</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>3000</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7">
+        <v>16</v>
+      </c>
+      <c r="C7">
+        <v>4800</v>
+      </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>18</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
We added support for testing external databases. TwoWaySQL module version 2.7.0 or later is required to test external databases.
</commit_message>
<xml_diff>
--- a/src/MxDBUnit/resources/mxdbunit/sample/sample1.xlsx
+++ b/src/MxDBUnit/resources/mxdbunit/sample/sample1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\MxDBUnit\src\MxDBUnit\resources\mxdbunit\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28357E7B-0E3F-4C92-BFB6-B4B6FBC439A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7766EAB-9309-4749-B8DB-7B213383C776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43824" yWindow="-4704" windowWidth="21864" windowHeight="10680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39492" yWindow="-5964" windowWidth="26736" windowHeight="18396" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="#ReadMe" sheetId="8" r:id="rId1"/>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="73">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1"/>
@@ -306,44 +306,272 @@
     <t>・MxDBUnitは"="で始まるシート名のシートを期待結果シートとみなして、アサート処理で使用します。</t>
   </si>
   <si>
+    <t>・MxDBUnit treats sheets with names starting with "#" as documentation and ignores them.</t>
+  </si>
+  <si>
+    <t>・MxDBUnit treats sheets with names starting with "=" as expected result sheets and uses them for assertion processing.</t>
+  </si>
+  <si>
+    <t>・Name setup sheets using the format "ModuleName.EntityName". For expected result sheets, prefix this name with "=". The module name can be omitted if the entity name is unique across the entire application.</t>
+  </si>
+  <si>
+    <t>・Enter a logical, unique ID (one that is intuitive to you) in the "Id" column. When loading entities, MxDBUnit builds an internal mapping between the logical IDs used in Excel and the physical IDs used in the database. This allows it to automatically convert logical IDs listed in association columns on subsequent sheets into physical IDs, thereby establishing entity associations. Therefore, please arrange your setup data sheets so that the entity being referenced by an association appears to the left of the referencing entity.</t>
+  </si>
+  <si>
+    <t>・期待結果シートで被テストロジックによって追加されたレコードをアサートしたい場合はレコードを特定するためヘッダーの列名に'*'をつけて下さい。複数の列を指定する事も出来ます。</t>
+  </si>
+  <si>
+    <t>・また、被テストロジックによって追加されたレコードについては、期待結果シートの'Id'列はブランクにして下さい。</t>
+  </si>
+  <si>
+    <t>・MxDBUnit treats sheets with names starting with characters other than "#" or "=" as setup data and uses them to load setup data.</t>
+  </si>
+  <si>
+    <t>・If you wish to assert records added by the logic under test in an expected result sheet, append an "*" to the header column name(s) used to identify the record. You may specify multiple columns.</t>
+  </si>
+  <si>
+    <t>・Additionally, for records added by the logic under test, leave the "Id" column blank in the expected result sheet.</t>
+  </si>
+  <si>
+    <t>・期待結果シートの"="以降が永続エンティティに該当しない場合はAssertAllByExcelアクションはそのシートをワーニングを出しつつスキップします。しかしAssertListByExcelアクションではシート名さえマッチすればそれがEntity名でなくてもアサートを実行します。</t>
+    <rPh sb="1" eb="3">
+      <t>キタイ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ケッカ</t>
+    </rPh>
+    <rPh sb="12" eb="14">
+      <t>イコウ</t>
+    </rPh>
+    <rPh sb="15" eb="17">
+      <t>エイゾク</t>
+    </rPh>
+    <rPh sb="24" eb="26">
+      <t>ガイトウ</t>
+    </rPh>
+    <rPh sb="29" eb="31">
+      <t>バアイ</t>
+    </rPh>
+    <rPh sb="66" eb="67">
+      <t>ダ</t>
+    </rPh>
+    <rPh sb="108" eb="109">
+      <t>メイ</t>
+    </rPh>
+    <rPh sb="126" eb="127">
+      <t>メイ</t>
+    </rPh>
+    <rPh sb="137" eb="139">
+      <t>ジッコウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>・If the text following the "=" sign in the "Expected Results" sheet does not correspond to a persistent entity, the **AssertAllByExcel** action skips that sheet while issuing a warning. In contrast, the **AssertListByExcel** action performs the assertion as long as the sheet name matches, even if it is not an entity name.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>・MxDBUnitは"#"と"="以外で始まるシート名のシートを準備データとみなして準備データのロードに使用します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>基本ルール</t>
+    <rPh sb="0" eb="2">
+      <t>キホン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>外部DBテストに関する追加ルール</t>
+    <rPh sb="0" eb="2">
+      <t>ガイブ</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>カン</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>ツイカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>・準備シートのシート名はモジュール名.エンティティ名として下さい。期待結果シートは、それに"="をつけて下さい。モジュール名はEntity名がアプリ全体で重複しなければ省略可能です。</t>
-  </si>
-  <si>
-    <t>・MxDBUnitは"#"と"="以外で始まるシート名のシートを準備データとみなして準備データのロードに使用します。</t>
-  </si>
-  <si>
-    <t>・MxDBUnit treats sheets with names starting with "#" as documentation and ignores them.</t>
-  </si>
-  <si>
-    <t>・MxDBUnit treats sheets with names starting with "=" as expected result sheets and uses them for assertion processing.</t>
-  </si>
-  <si>
-    <t>・Name setup sheets using the format "ModuleName.EntityName". For expected result sheets, prefix this name with "=". The module name can be omitted if the entity name is unique across the entire application.</t>
-  </si>
-  <si>
-    <t>・Enter a logical, unique ID (one that is intuitive to you) in the "Id" column. When loading entities, MxDBUnit builds an internal mapping between the logical IDs used in Excel and the physical IDs used in the database. This allows it to automatically convert logical IDs listed in association columns on subsequent sheets into physical IDs, thereby establishing entity associations. Therefore, please arrange your setup data sheets so that the entity being referenced by an association appears to the left of the referencing entity.</t>
-  </si>
-  <si>
-    <t>・期待結果シートで被テストロジックによって追加されたレコードをアサートしたい場合はレコードを特定するためヘッダーの列名に'*'をつけて下さい。複数の列を指定する事も出来ます。</t>
-  </si>
-  <si>
-    <t>・また、被テストロジックによって追加されたレコードについては、期待結果シートの'Id'列はブランクにして下さい。</t>
-  </si>
-  <si>
-    <t>・MxDBUnit treats sheets with names starting with characters other than "#" or "=" as setup data and uses them to load setup data.</t>
-  </si>
-  <si>
-    <t>・If you wish to assert records added by the logic under test in an expected result sheet, append an "*" to the header column name(s) used to identify the record. You may specify multiple columns.</t>
-  </si>
-  <si>
-    <t>・Additionally, for records added by the logic under test, leave the "Id" column blank in the expected result sheet.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>・１つのテストで内部DBと外部DBの両方を扱う事が可能です。</t>
+    <rPh sb="8" eb="10">
+      <t>ナイブ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>ガイブ</t>
+    </rPh>
+    <rPh sb="18" eb="20">
+      <t>リョウホウ</t>
+    </rPh>
+    <rPh sb="21" eb="22">
+      <t>アツカ</t>
+    </rPh>
+    <rPh sb="23" eb="24">
+      <t>コト</t>
+    </rPh>
+    <rPh sb="25" eb="27">
+      <t>カノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>・外部DBの場合は内部DBと異なり"Id"列は特別な意味を持ちません。そのため期待結果シートではキー列の列名に"*"が必ず必要となります。キー列が指定されていないと正しくアサートが行われません。</t>
+    <rPh sb="1" eb="3">
+      <t>ガイブ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>バアイ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>ナイブ</t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t>コト</t>
+    </rPh>
+    <rPh sb="21" eb="22">
+      <t>レツ</t>
+    </rPh>
+    <rPh sb="23" eb="25">
+      <t>トクベツ</t>
+    </rPh>
+    <rPh sb="26" eb="28">
+      <t>イミ</t>
+    </rPh>
+    <rPh sb="29" eb="30">
+      <t>モ</t>
+    </rPh>
+    <rPh sb="39" eb="41">
+      <t>キタイ</t>
+    </rPh>
+    <rPh sb="41" eb="43">
+      <t>ケッカ</t>
+    </rPh>
+    <rPh sb="50" eb="51">
+      <t>レツ</t>
+    </rPh>
+    <rPh sb="52" eb="53">
+      <t>レツ</t>
+    </rPh>
+    <rPh sb="53" eb="54">
+      <t>メイ</t>
+    </rPh>
+    <rPh sb="59" eb="60">
+      <t>カナラ</t>
+    </rPh>
+    <rPh sb="61" eb="63">
+      <t>ヒツヨウ</t>
+    </rPh>
+    <rPh sb="71" eb="72">
+      <t>レツ</t>
+    </rPh>
+    <rPh sb="73" eb="75">
+      <t>シテイ</t>
+    </rPh>
+    <rPh sb="82" eb="83">
+      <t>タダ</t>
+    </rPh>
+    <rPh sb="90" eb="91">
+      <t>オコナ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>・外部DBテストの場合は、準備シートのシート名は、"TwoWaySQLモジュールの外部データソース名|テーブル名"（Ex. "EXTDS|EMPLOYEE"）として下さい。期待結果シートは、それに"="をつけて下さい。</t>
+    <rPh sb="1" eb="3">
+      <t>ガイブ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>バアイ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>ジュンビ</t>
+    </rPh>
+    <rPh sb="22" eb="23">
+      <t>メイ</t>
+    </rPh>
+    <rPh sb="41" eb="43">
+      <t>ガイブ</t>
+    </rPh>
+    <rPh sb="49" eb="50">
+      <t>メイ</t>
+    </rPh>
+    <rPh sb="55" eb="56">
+      <t>メイ</t>
+    </rPh>
+    <rPh sb="82" eb="83">
+      <t>クダ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Additional rules for external DB testing:</t>
+  </si>
+  <si>
+    <t>・For external DB tests, name the preparation sheet using the format "TwoWaySQL module's external data source name|table name" (e.g., "EXTDS|EMPLOYEE"). For the expected results sheet, prefix that name with "=".</t>
+  </si>
+  <si>
+    <t>・Unlike internal DBs, the "Id" column holds no special significance for external DBs. Therefore, you must include an "*" in the column name of the key column within the expected results sheet. If a key column is not specified, assertions will not be performed correctly.</t>
+  </si>
+  <si>
+    <t>・A single test can handle both internal and external databases.</t>
+  </si>
+  <si>
+    <t>Basic Rules:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>・外部DBのテストを行う場合は必ずテストケースのMicroflowのあるモジュールに"TearDown" Microflowを作成して"TearDownMxDBUnit" Actionを呼び出して下さい。これはデッドロック回避のための必須要件です。</t>
+    <rPh sb="1" eb="3">
+      <t>ガイブ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>オコナ</t>
+    </rPh>
+    <rPh sb="12" eb="14">
+      <t>バアイ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>カナラ</t>
+    </rPh>
+    <rPh sb="63" eb="65">
+      <t>サクセイ</t>
+    </rPh>
+    <rPh sb="93" eb="94">
+      <t>ヨ</t>
+    </rPh>
+    <rPh sb="95" eb="96">
+      <t>ダ</t>
+    </rPh>
+    <rPh sb="98" eb="99">
+      <t>クダ</t>
+    </rPh>
+    <rPh sb="111" eb="113">
+      <t>カイヒ</t>
+    </rPh>
+    <rPh sb="117" eb="119">
+      <t>ヒッス</t>
+    </rPh>
+    <rPh sb="119" eb="121">
+      <t>ヨウケン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>・When testing an external DB, you must create a "TearDown" Microflow in the module containing the test case's Microflow and call the "TearDownMxDBUnit" action. This is a mandatory requirement to prevent deadlocks.</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -373,6 +601,13 @@
       <family val="3"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -394,8 +629,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -676,97 +912,167 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6F197F3-729B-4E7B-9286-490FA86AAF98}">
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
-        <v>50</v>
+    <row r="1" spans="1:1" ht="28.8">
+      <c r="A1" s="1" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:1">
-      <c r="A12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" t="s">
-        <v>47</v>
+    <row r="13" spans="1:1" ht="28.8">
+      <c r="A13" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="28.8">
+      <c r="A20" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:1">
-      <c r="A18" t="s">
+    <row r="27" spans="1:1">
+      <c r="A27" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
-      <c r="A19" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1">
-      <c r="A20" t="s">
-        <v>55</v>
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="28.8">
+      <c r="A32" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added an alias feature for table and entity names.
</commit_message>
<xml_diff>
--- a/src/MxDBUnit/resources/mxdbunit/sample/sample1.xlsx
+++ b/src/MxDBUnit/resources/mxdbunit/sample/sample1.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\MxDBUnit\src\MxDBUnit\resources\mxdbunit\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7766EAB-9309-4749-B8DB-7B213383C776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40E9D98C-456A-46B6-8253-AB5BFECF6502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39492" yWindow="-5964" windowWidth="26736" windowHeight="18396" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40284" yWindow="-4524" windowWidth="21744" windowHeight="10188" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="#ReadMe" sheetId="8" r:id="rId1"/>
-    <sheet name="MxDBUnit.Item" sheetId="1" r:id="rId2"/>
-    <sheet name="MxDBUnit.Customer" sheetId="4" r:id="rId3"/>
-    <sheet name="MxDBUnit.Order" sheetId="2" r:id="rId4"/>
-    <sheet name="MxDBUnit.OrderItem" sheetId="3" r:id="rId5"/>
-    <sheet name="=MxDBUnit.Customer" sheetId="5" r:id="rId6"/>
-    <sheet name="=MxDBUnit.Order" sheetId="6" r:id="rId7"/>
-    <sheet name="=MxDBUnit.OrderItem" sheetId="7" r:id="rId8"/>
+    <sheet name="#Alias" sheetId="9" r:id="rId2"/>
+    <sheet name="MxDBUnit.Item" sheetId="1" r:id="rId3"/>
+    <sheet name="MxDBUnit.Customer" sheetId="4" r:id="rId4"/>
+    <sheet name="MxDBUnit.Order" sheetId="2" r:id="rId5"/>
+    <sheet name="MxDBUnit.OrderItem" sheetId="3" r:id="rId6"/>
+    <sheet name="=MxDBUnit.Customer" sheetId="5" r:id="rId7"/>
+    <sheet name="=MxDBUnit.Order" sheetId="6" r:id="rId8"/>
+    <sheet name="=MxDBUnit.OrderItem" sheetId="7" r:id="rId9"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -32,6 +33,33 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>suzuki yuta</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{B7BA362E-D960-41B4-B5E6-871B39212050}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="MS P ゴシック"/>
+            <family val="3"/>
+            <charset val="128"/>
+          </rPr>
+          <t>If an entity name or table name is too long to be used as a sheet name, you can specify a shortened name in the AliasName field and the actual name in the OriginalName field; the conversion will then be performed at runtime.
+For an external database, specify only the table name in the AliasName field.
+For an internal database, match the inclusion or exclusion of the module name to the sheet name.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>suzuki yuta</author>
@@ -81,7 +109,7 @@
 </comments>
 </file>
 
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>suzuki yuta</author>
@@ -119,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="75">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1"/>
@@ -564,6 +592,14 @@
   </si>
   <si>
     <t>・When testing an external DB, you must create a "TearDown" Microflow in the module containing the test case's Microflow and call the "TearDownMxDBUnit" action. This is a mandatory requirement to prevent deadlocks.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>OriginalName</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AliasName</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1082,6 +1118,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7EA9907-35FC-4D16-B4C0-867B27B45C6E}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.69921875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -1152,7 +1212,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AEE99C2-9E27-465E-B6CB-6A2D58F84035}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -1211,7 +1271,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A53E7E-2292-455C-86A3-346B7EDF246B}">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -1298,7 +1358,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EC0B6D4-E629-427B-86DA-8D931806A50F}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -1435,7 +1495,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05855E9E-4A78-4337-A1E6-41A1A78B0F61}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -1494,7 +1554,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A7D26DE-4B43-4B1A-96E5-470F26423CE2}">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="18"/>
@@ -1581,7 +1641,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA993482-7DB0-4E07-A12A-DB0076CC842D}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="18"/>

</xml_diff>